<commit_message>
Update Short Semester I (E24 Batch).xlsx
</commit_message>
<xml_diff>
--- a/Short Semester I (E24 Batch).xlsx
+++ b/Short Semester I (E24 Batch).xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\theva\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maids.jfn\Documents\GitHub\MC3020_Attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A51ED7CA-EA5E-4948-9CC4-917249FF1C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="MC9030" sheetId="2" r:id="rId1"/>
@@ -2164,7 +2163,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2314,7 +2313,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -2559,6 +2558,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2568,7 +2578,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2759,14 +2769,17 @@
     <xf numFmtId="2" fontId="22" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 15" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal_Sheet1" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Normal_Sheet1_1" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 15" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="3"/>
+    <cellStyle name="Normal 2 2" xfId="4"/>
+    <cellStyle name="Normal_Sheet1" xfId="1"/>
+    <cellStyle name="Normal_Sheet1_1" xfId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3043,7 +3056,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G210"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7466,7 +7479,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G178"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
@@ -11228,8 +11241,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G122"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" customWidth="1"/>
@@ -13805,13 +13818,16 @@
       </c>
       <c r="G122" s="68"/>
     </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" s="70"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G198"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -17916,7 +17932,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB6E2A7E-2D4B-4BFC-938E-45B79060EAA5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G177"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -20379,17 +20395,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2835d969-06cc-46e6-b4cc-c525f784ce43">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="03c84e3c-1549-479a-8619-e0d964aa7481" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100455C4072EA7E0D46870C67AD0D3E62C3" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6d62d4992a7888825600c982e6c75641">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2835d969-06cc-46e6-b4cc-c525f784ce43" xmlns:ns3="03c84e3c-1549-479a-8619-e0d964aa7481" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9015832621b6abd41b87bce5adc31c29" ns2:_="" ns3:_="">
     <xsd:import namespace="2835d969-06cc-46e6-b4cc-c525f784ce43"/>
@@ -20644,7 +20649,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -20653,24 +20658,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA8EACE5-8C5B-48FA-AFAD-2C86FB600767}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2835d969-06cc-46e6-b4cc-c525f784ce43"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="03c84e3c-1549-479a-8619-e0d964aa7481"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2835d969-06cc-46e6-b4cc-c525f784ce43">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="03c84e3c-1549-479a-8619-e0d964aa7481" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46A244EB-A970-4F2B-8B12-6A24EFA3E1AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20689,10 +20688,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{781D7AC4-6CC5-4242-91F0-BEE6E1ED618F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA8EACE5-8C5B-48FA-AFAD-2C86FB600767}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2835d969-06cc-46e6-b4cc-c525f784ce43"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="03c84e3c-1549-479a-8619-e0d964aa7481"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>